<commit_message>
Add new files and  remake old
</commit_message>
<xml_diff>
--- a/Эксп.техн.ср.движ.поездов_(Фадеев_К.С.)/Курсавая.xlsx
+++ b/Эксп.техн.ср.движ.поездов_(Фадеев_К.С.)/Курсавая.xlsx
@@ -8,24 +8,37 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Github\3Course-\Эксп.техн.ср.движ.поездов_(Фадеев_К.С.)\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E9E40309-B3F4-4792-A67B-C7DC6ADEFF9D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{269B75D0-153F-487E-8C01-5608554E1EDF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
+    <sheet name="Sheet3" sheetId="3" r:id="rId3"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="72" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="135" uniqueCount="60">
   <si>
     <t>Обслуживание устройства цифровая</t>
   </si>
@@ -151,13 +164,67 @@
   </si>
   <si>
     <t>.5/2</t>
+  </si>
+  <si>
+    <t>Факсимильные телеграфные аппараты, аппарат</t>
+  </si>
+  <si>
+    <t>0/550</t>
+  </si>
+  <si>
+    <t>Оборудование</t>
+  </si>
+  <si>
+    <t>Количество оборудования на станции, расположенной на линии категории</t>
+  </si>
+  <si>
+    <t>I</t>
+  </si>
+  <si>
+    <t>II</t>
+  </si>
+  <si>
+    <t>III</t>
+  </si>
+  <si>
+    <t>IV</t>
+  </si>
+  <si>
+    <t>Аппаратура ВЧ телефония:</t>
+  </si>
+  <si>
+    <t>Цифровые оконечные оконченные полукомплекты,канал.</t>
+  </si>
+  <si>
+    <t>Аналоговые оконечные оконченные полукомплекты,канал.</t>
+  </si>
+  <si>
+    <t>Распорядительные станции подстанционной связи, комплект</t>
+  </si>
+  <si>
+    <t>Телефонные аппараты, аппарат</t>
+  </si>
+  <si>
+    <t>Промежуточные пункты ОТС,промпункт</t>
+  </si>
+  <si>
+    <t>Аппаратура связи совещаний на станциях, комплект</t>
+  </si>
+  <si>
+    <t>Радиостанции стационарные ПРС, р/ст</t>
+  </si>
+  <si>
+    <t>Радиостанции стационарные СРС, р/ст</t>
+  </si>
+  <si>
+    <t>Аппаратура регестрации служебных переговоров, комплект</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -177,8 +244,15 @@
       <name val="Times New Roman"/>
       <family val="1"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="5">
+  <fills count="7">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -203,8 +277,20 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFD0CECE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFFF"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="15">
+  <borders count="16">
     <border>
       <left/>
       <right/>
@@ -370,11 +456,22 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="30">
+  <cellXfs count="56">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -397,54 +494,126 @@
     <xf numFmtId="12" fontId="2" fillId="2" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="16" fontId="2" fillId="2" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="8"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -800,32 +969,32 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:18" ht="75.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="11" t="s">
+      <c r="A1" s="26" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="12" t="s">
+      <c r="B1" s="9" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="17" t="s">
+      <c r="C1" s="12" t="s">
         <v>2</v>
       </c>
-      <c r="H1" s="15" t="s">
+      <c r="H1" s="8" t="s">
         <v>0</v>
       </c>
-      <c r="I1" s="12" t="s">
+      <c r="I1" s="9" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="2" spans="1:18" ht="56.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="13"/>
-      <c r="B2" s="14">
+      <c r="A2" s="27"/>
+      <c r="B2" s="11">
         <v>7</v>
       </c>
-      <c r="C2" s="18">
+      <c r="C2" s="13">
         <v>7</v>
       </c>
-      <c r="H2" s="16"/>
-      <c r="I2" s="14">
+      <c r="H2" s="10"/>
+      <c r="I2" s="11">
         <v>7</v>
       </c>
     </row>
@@ -847,31 +1016,31 @@
       </c>
     </row>
     <row r="4" spans="1:18" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="8" t="s">
+      <c r="A4" s="24" t="s">
         <v>3</v>
       </c>
-      <c r="B4" s="10"/>
-      <c r="C4" s="9"/>
-      <c r="E4" s="8" t="s">
+      <c r="B4" s="28"/>
+      <c r="C4" s="25"/>
+      <c r="E4" s="24" t="s">
         <v>14</v>
       </c>
-      <c r="F4" s="9"/>
-      <c r="H4" s="8" t="s">
+      <c r="F4" s="25"/>
+      <c r="H4" s="24" t="s">
         <v>3</v>
       </c>
-      <c r="I4" s="9"/>
-      <c r="K4" s="8" t="s">
+      <c r="I4" s="25"/>
+      <c r="K4" s="24" t="s">
         <v>22</v>
       </c>
-      <c r="L4" s="9"/>
-      <c r="N4" s="8" t="s">
+      <c r="L4" s="25"/>
+      <c r="N4" s="24" t="s">
         <v>14</v>
       </c>
-      <c r="O4" s="9"/>
-      <c r="Q4" s="8" t="s">
+      <c r="O4" s="25"/>
+      <c r="Q4" s="24" t="s">
         <v>26</v>
       </c>
-      <c r="R4" s="9"/>
+      <c r="R4" s="25"/>
     </row>
     <row r="5" spans="1:18" ht="37.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A5" s="3" t="s">
@@ -1018,10 +1187,10 @@
       <c r="I8" s="1">
         <v>19</v>
       </c>
-      <c r="K8" s="8" t="s">
+      <c r="K8" s="24" t="s">
         <v>26</v>
       </c>
-      <c r="L8" s="9"/>
+      <c r="L8" s="25"/>
       <c r="N8" s="3" t="s">
         <v>19</v>
       </c>
@@ -1098,14 +1267,14 @@
       <c r="L10" s="1">
         <v>3</v>
       </c>
-      <c r="N10" s="8" t="s">
+      <c r="N10" s="24" t="s">
         <v>22</v>
       </c>
-      <c r="O10" s="9"/>
-      <c r="Q10" s="11" t="s">
+      <c r="O10" s="25"/>
+      <c r="Q10" s="26" t="s">
         <v>33</v>
       </c>
-      <c r="R10" s="12" t="s">
+      <c r="R10" s="9" t="s">
         <v>34</v>
       </c>
     </row>
@@ -1113,10 +1282,10 @@
       <c r="A11" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="B11" s="19" t="s">
+      <c r="B11" s="14" t="s">
         <v>12</v>
       </c>
-      <c r="C11" s="20" t="s">
+      <c r="C11" s="15" t="s">
         <v>13</v>
       </c>
       <c r="H11" s="3" t="s">
@@ -1137,17 +1306,17 @@
       <c r="O11" s="1">
         <v>37</v>
       </c>
-      <c r="Q11" s="13"/>
-      <c r="R11" s="14">
+      <c r="Q11" s="27"/>
+      <c r="R11" s="11">
         <v>7</v>
       </c>
     </row>
     <row r="12" spans="1:18" ht="38.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B12" s="21"/>
-      <c r="C12" s="22"/>
-      <c r="D12" s="22"/>
-      <c r="E12" s="22"/>
-      <c r="F12" s="23"/>
+      <c r="B12" s="16"/>
+      <c r="C12" s="17"/>
+      <c r="D12" s="17"/>
+      <c r="E12" s="17"/>
+      <c r="F12" s="18"/>
       <c r="K12" s="3" t="s">
         <v>30</v>
       </c>
@@ -1168,11 +1337,8 @@
       </c>
     </row>
     <row r="13" spans="1:18" ht="38.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B13" s="24"/>
-      <c r="C13" s="25"/>
-      <c r="D13" s="25"/>
-      <c r="E13" s="25"/>
-      <c r="F13" s="26"/>
+      <c r="B13" s="19"/>
+      <c r="F13" s="20"/>
       <c r="K13" s="3" t="s">
         <v>32</v>
       </c>
@@ -1193,11 +1359,8 @@
       </c>
     </row>
     <row r="14" spans="1:18" ht="38.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B14" s="24"/>
-      <c r="C14" s="25"/>
-      <c r="D14" s="25"/>
-      <c r="E14" s="25"/>
-      <c r="F14" s="26"/>
+      <c r="B14" s="19"/>
+      <c r="F14" s="20"/>
       <c r="Q14" s="5" t="s">
         <v>37</v>
       </c>
@@ -1206,11 +1369,11 @@
       </c>
     </row>
     <row r="15" spans="1:18" ht="57" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B15" s="27"/>
-      <c r="C15" s="28"/>
-      <c r="D15" s="28"/>
-      <c r="E15" s="28"/>
-      <c r="F15" s="29"/>
+      <c r="B15" s="21"/>
+      <c r="C15" s="22"/>
+      <c r="D15" s="22"/>
+      <c r="E15" s="22"/>
+      <c r="F15" s="23"/>
       <c r="Q15" s="5" t="s">
         <v>38</v>
       </c>
@@ -1222,18 +1385,814 @@
     <row r="60" ht="78" customHeight="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <mergeCells count="10">
+    <mergeCell ref="A1:A2"/>
+    <mergeCell ref="A4:C4"/>
+    <mergeCell ref="K4:L4"/>
+    <mergeCell ref="H4:I4"/>
     <mergeCell ref="E4:F4"/>
     <mergeCell ref="K8:L8"/>
     <mergeCell ref="N4:O4"/>
     <mergeCell ref="N10:O10"/>
     <mergeCell ref="Q4:R4"/>
     <mergeCell ref="Q10:Q11"/>
-    <mergeCell ref="A1:A2"/>
-    <mergeCell ref="A4:C4"/>
-    <mergeCell ref="K4:L4"/>
-    <mergeCell ref="H4:I4"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4ABDF1AB-B0DE-43D8-B9A0-8E05EC648D9C}">
+  <dimension ref="A1:I39"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="34.140625" customWidth="1"/>
+    <col min="2" max="2" width="23.28515625" customWidth="1"/>
+    <col min="3" max="3" width="13.28515625" customWidth="1"/>
+    <col min="9" max="9" width="12.85546875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="2" spans="1:9" ht="57" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="33" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" s="30" t="s">
+        <v>1</v>
+      </c>
+      <c r="C2" s="31" t="s">
+        <v>2</v>
+      </c>
+      <c r="D2" s="40"/>
+      <c r="E2" s="54"/>
+      <c r="F2" s="54"/>
+      <c r="G2" s="54"/>
+      <c r="H2" s="54"/>
+      <c r="I2" s="54"/>
+    </row>
+    <row r="3" spans="1:9" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="29"/>
+      <c r="B3" s="1">
+        <v>7</v>
+      </c>
+      <c r="C3" s="2">
+        <v>7</v>
+      </c>
+      <c r="D3" s="40"/>
+      <c r="E3" s="55"/>
+      <c r="F3" s="55"/>
+      <c r="G3" s="55"/>
+      <c r="H3" s="55"/>
+      <c r="I3" s="54"/>
+    </row>
+    <row r="4" spans="1:9" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="3">
+        <v>1</v>
+      </c>
+      <c r="B4" s="1">
+        <v>8</v>
+      </c>
+      <c r="C4" s="2">
+        <v>8</v>
+      </c>
+      <c r="D4" s="40"/>
+      <c r="E4" s="55"/>
+      <c r="F4" s="55"/>
+      <c r="G4" s="55"/>
+      <c r="H4" s="55"/>
+      <c r="I4" s="55"/>
+    </row>
+    <row r="5" spans="1:9" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="36" t="s">
+        <v>3</v>
+      </c>
+      <c r="B5" s="37"/>
+      <c r="C5" s="32"/>
+      <c r="D5" s="40"/>
+      <c r="E5" s="50"/>
+      <c r="F5" s="50"/>
+      <c r="G5" s="50"/>
+      <c r="H5" s="50"/>
+      <c r="I5" s="55"/>
+    </row>
+    <row r="6" spans="1:9" ht="58.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="49" t="s">
+        <v>4</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="D6" s="39"/>
+      <c r="E6" s="50"/>
+      <c r="F6" s="50"/>
+      <c r="G6" s="51"/>
+      <c r="H6" s="51"/>
+      <c r="I6" s="52"/>
+    </row>
+    <row r="7" spans="1:9" ht="57" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="49" t="s">
+        <v>7</v>
+      </c>
+      <c r="B7" s="1">
+        <v>570</v>
+      </c>
+      <c r="C7" s="2">
+        <v>270</v>
+      </c>
+      <c r="D7" s="39"/>
+      <c r="E7" s="50"/>
+      <c r="F7" s="50"/>
+      <c r="G7" s="51"/>
+      <c r="H7" s="51"/>
+      <c r="I7" s="52"/>
+    </row>
+    <row r="8" spans="1:9" ht="36.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="49" t="s">
+        <v>8</v>
+      </c>
+      <c r="B8" s="1">
+        <v>7900</v>
+      </c>
+      <c r="C8" s="2">
+        <v>2900</v>
+      </c>
+      <c r="D8" s="39"/>
+      <c r="E8" s="50"/>
+      <c r="F8" s="50"/>
+      <c r="G8" s="51"/>
+      <c r="H8" s="51"/>
+      <c r="I8" s="52"/>
+    </row>
+    <row r="9" spans="1:9" ht="35.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A9" s="49" t="s">
+        <v>42</v>
+      </c>
+      <c r="B9" s="1">
+        <v>43</v>
+      </c>
+      <c r="C9" s="2">
+        <v>19</v>
+      </c>
+      <c r="D9" s="39"/>
+      <c r="E9" s="50"/>
+      <c r="F9" s="50"/>
+      <c r="G9" s="51"/>
+      <c r="H9" s="51"/>
+      <c r="I9" s="52"/>
+    </row>
+    <row r="10" spans="1:9" ht="75.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A10" s="49" t="s">
+        <v>9</v>
+      </c>
+      <c r="B10" s="4" t="s">
+        <v>41</v>
+      </c>
+      <c r="C10" s="35" t="s">
+        <v>40</v>
+      </c>
+      <c r="D10" s="39"/>
+      <c r="E10" s="50"/>
+      <c r="F10" s="50"/>
+      <c r="G10" s="51"/>
+      <c r="H10" s="51"/>
+      <c r="I10" s="52"/>
+    </row>
+    <row r="11" spans="1:9" ht="57" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A11" s="49" t="s">
+        <v>10</v>
+      </c>
+      <c r="B11" s="1">
+        <v>800</v>
+      </c>
+      <c r="C11" s="2">
+        <v>900</v>
+      </c>
+      <c r="D11" s="39"/>
+      <c r="E11" s="50"/>
+      <c r="F11" s="50"/>
+      <c r="G11" s="51"/>
+      <c r="H11" s="51"/>
+      <c r="I11" s="52"/>
+    </row>
+    <row r="12" spans="1:9" ht="57" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A12" s="49" t="s">
+        <v>11</v>
+      </c>
+      <c r="B12" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="C12" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D12" s="39"/>
+      <c r="E12" s="50"/>
+      <c r="F12" s="50"/>
+      <c r="G12" s="51"/>
+      <c r="H12" s="51"/>
+      <c r="I12" s="52"/>
+    </row>
+    <row r="13" spans="1:9" ht="18.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A13" s="36" t="s">
+        <v>14</v>
+      </c>
+      <c r="B13" s="37"/>
+      <c r="C13" s="32"/>
+      <c r="D13" s="39"/>
+      <c r="E13" s="50"/>
+      <c r="F13" s="53"/>
+      <c r="G13" s="52"/>
+      <c r="H13" s="52"/>
+      <c r="I13" s="52"/>
+    </row>
+    <row r="14" spans="1:9" ht="75.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A14" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="B14" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="C14" s="41" t="s">
+        <v>16</v>
+      </c>
+      <c r="D14" s="39"/>
+      <c r="E14" s="50"/>
+      <c r="F14" s="53"/>
+      <c r="G14" s="52"/>
+      <c r="H14" s="52"/>
+      <c r="I14" s="52"/>
+    </row>
+    <row r="15" spans="1:9" ht="44.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A15" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="B15" s="1">
+        <v>89</v>
+      </c>
+      <c r="C15" s="41">
+        <v>45</v>
+      </c>
+      <c r="D15" s="39"/>
+      <c r="E15" s="50"/>
+      <c r="F15" s="53"/>
+      <c r="G15" s="52"/>
+      <c r="H15" s="52"/>
+      <c r="I15" s="52"/>
+    </row>
+    <row r="16" spans="1:9" ht="57.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A16" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="B16" s="1">
+        <v>29</v>
+      </c>
+      <c r="C16" s="41">
+        <v>13</v>
+      </c>
+      <c r="D16" s="39"/>
+      <c r="E16" s="50"/>
+      <c r="F16" s="53"/>
+      <c r="G16" s="52"/>
+      <c r="H16" s="52"/>
+      <c r="I16" s="52"/>
+    </row>
+    <row r="17" spans="1:9" ht="75.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A17" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="B17" s="1">
+        <v>85</v>
+      </c>
+      <c r="C17" s="41">
+        <v>46</v>
+      </c>
+      <c r="D17" s="39"/>
+      <c r="E17" s="50"/>
+      <c r="F17" s="53"/>
+      <c r="G17" s="52"/>
+      <c r="H17" s="52"/>
+      <c r="I17" s="52"/>
+    </row>
+    <row r="18" spans="1:9" ht="38.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A18" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="B18" s="1">
+        <v>53</v>
+      </c>
+      <c r="C18" s="41">
+        <v>26</v>
+      </c>
+      <c r="D18" s="39"/>
+      <c r="E18" s="50"/>
+      <c r="F18" s="53"/>
+      <c r="G18" s="52"/>
+      <c r="H18" s="52"/>
+      <c r="I18" s="52"/>
+    </row>
+    <row r="19" spans="1:9" ht="30.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A19" s="36" t="s">
+        <v>22</v>
+      </c>
+      <c r="B19" s="37"/>
+      <c r="C19" s="32"/>
+      <c r="D19" s="38"/>
+      <c r="E19" s="50"/>
+      <c r="F19" s="53"/>
+      <c r="G19" s="52"/>
+      <c r="H19" s="52"/>
+      <c r="I19" s="52"/>
+    </row>
+    <row r="20" spans="1:9" ht="57" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A20" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="B20" s="1">
+        <v>74</v>
+      </c>
+      <c r="C20" s="41">
+        <v>37</v>
+      </c>
+      <c r="D20" s="38"/>
+      <c r="E20" s="50"/>
+      <c r="F20" s="53"/>
+      <c r="G20" s="52"/>
+      <c r="H20" s="52"/>
+      <c r="I20" s="52"/>
+    </row>
+    <row r="21" spans="1:9" ht="57" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A21" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="B21" s="1">
+        <v>35</v>
+      </c>
+      <c r="C21" s="41">
+        <v>17</v>
+      </c>
+      <c r="D21" s="38"/>
+      <c r="E21" s="50"/>
+      <c r="F21" s="53"/>
+      <c r="G21" s="52"/>
+      <c r="H21" s="52"/>
+      <c r="I21" s="52"/>
+    </row>
+    <row r="22" spans="1:9" ht="57" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A22" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="B22" s="1">
+        <v>86</v>
+      </c>
+      <c r="C22" s="41">
+        <v>43</v>
+      </c>
+      <c r="E22" s="50"/>
+      <c r="F22" s="52"/>
+      <c r="G22" s="52"/>
+      <c r="H22" s="52"/>
+      <c r="I22" s="52"/>
+    </row>
+    <row r="23" spans="1:9" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A23" s="36" t="s">
+        <v>26</v>
+      </c>
+      <c r="B23" s="37"/>
+      <c r="C23" s="32"/>
+      <c r="E23" s="50"/>
+      <c r="F23" s="52"/>
+      <c r="G23" s="52"/>
+      <c r="H23" s="52"/>
+      <c r="I23" s="52"/>
+    </row>
+    <row r="24" spans="1:9" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A24" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="B24" s="1">
+        <v>33</v>
+      </c>
+      <c r="C24" s="41">
+        <v>16</v>
+      </c>
+      <c r="E24" s="50"/>
+      <c r="F24" s="52"/>
+      <c r="G24" s="52"/>
+      <c r="H24" s="52"/>
+      <c r="I24" s="52"/>
+    </row>
+    <row r="25" spans="1:9" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A25" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="B25" s="1">
+        <v>5</v>
+      </c>
+      <c r="C25" s="41">
+        <v>3</v>
+      </c>
+      <c r="E25" s="50"/>
+      <c r="F25" s="52"/>
+      <c r="G25" s="52"/>
+      <c r="H25" s="52"/>
+      <c r="I25" s="52"/>
+    </row>
+    <row r="26" spans="1:9" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A26" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="B26" s="1">
+        <v>21</v>
+      </c>
+      <c r="C26" s="41">
+        <v>11</v>
+      </c>
+      <c r="E26" s="50"/>
+      <c r="F26" s="52"/>
+      <c r="G26" s="52"/>
+      <c r="H26" s="52"/>
+      <c r="I26" s="52"/>
+    </row>
+    <row r="27" spans="1:9" ht="38.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A27" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="B27" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="C27" s="41" t="s">
+        <v>31</v>
+      </c>
+      <c r="E27" s="50"/>
+      <c r="F27" s="52"/>
+      <c r="G27" s="52"/>
+      <c r="H27" s="52"/>
+      <c r="I27" s="52"/>
+    </row>
+    <row r="28" spans="1:9" ht="38.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A28" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="B28" s="1">
+        <v>13</v>
+      </c>
+      <c r="C28" s="41">
+        <v>7</v>
+      </c>
+      <c r="E28" s="50"/>
+      <c r="F28" s="52"/>
+      <c r="G28" s="52"/>
+      <c r="H28" s="52"/>
+      <c r="I28" s="52"/>
+    </row>
+    <row r="29" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="E29" s="50"/>
+      <c r="F29" s="52"/>
+      <c r="G29" s="52"/>
+      <c r="H29" s="52"/>
+      <c r="I29" s="52"/>
+    </row>
+    <row r="30" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="E30" s="50"/>
+      <c r="F30" s="52"/>
+      <c r="G30" s="52"/>
+      <c r="H30" s="52"/>
+      <c r="I30" s="52"/>
+    </row>
+    <row r="31" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="E31" s="50"/>
+      <c r="F31" s="52"/>
+      <c r="G31" s="52"/>
+      <c r="H31" s="52"/>
+      <c r="I31" s="52"/>
+    </row>
+    <row r="32" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="E32" s="50"/>
+      <c r="F32" s="52"/>
+      <c r="G32" s="52"/>
+      <c r="H32" s="52"/>
+      <c r="I32" s="52"/>
+    </row>
+    <row r="33" spans="5:9" x14ac:dyDescent="0.25">
+      <c r="E33" s="50"/>
+      <c r="F33" s="52"/>
+      <c r="G33" s="52"/>
+      <c r="H33" s="52"/>
+      <c r="I33" s="52"/>
+    </row>
+    <row r="34" spans="5:9" x14ac:dyDescent="0.25">
+      <c r="E34" s="50"/>
+      <c r="F34" s="52"/>
+      <c r="G34" s="52"/>
+      <c r="H34" s="52"/>
+      <c r="I34" s="52"/>
+    </row>
+    <row r="35" spans="5:9" x14ac:dyDescent="0.25">
+      <c r="E35" s="50"/>
+      <c r="F35" s="52"/>
+      <c r="G35" s="52"/>
+      <c r="H35" s="52"/>
+      <c r="I35" s="52"/>
+    </row>
+    <row r="36" spans="5:9" x14ac:dyDescent="0.25">
+      <c r="E36" s="50"/>
+      <c r="F36" s="52"/>
+      <c r="G36" s="52"/>
+      <c r="H36" s="52"/>
+      <c r="I36" s="52"/>
+    </row>
+    <row r="37" spans="5:9" x14ac:dyDescent="0.25">
+      <c r="E37" s="50"/>
+      <c r="F37" s="52"/>
+      <c r="G37" s="52"/>
+      <c r="H37" s="52"/>
+      <c r="I37" s="52"/>
+    </row>
+    <row r="38" spans="5:9" x14ac:dyDescent="0.25">
+      <c r="E38" s="50"/>
+      <c r="F38" s="52"/>
+      <c r="G38" s="52"/>
+      <c r="H38" s="52"/>
+      <c r="I38" s="52"/>
+    </row>
+    <row r="39" spans="5:9" x14ac:dyDescent="0.25">
+      <c r="E39" s="50"/>
+      <c r="F39" s="52"/>
+      <c r="G39" s="52"/>
+      <c r="H39" s="52"/>
+      <c r="I39" s="52"/>
+    </row>
+  </sheetData>
+  <mergeCells count="5">
+    <mergeCell ref="A19:C19"/>
+    <mergeCell ref="A23:C23"/>
+    <mergeCell ref="A2:A3"/>
+    <mergeCell ref="A5:C5"/>
+    <mergeCell ref="A13:C13"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7AA66622-1F0D-4754-9BCA-24802D860A68}">
+  <dimension ref="A1:E19"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="56.7109375" customWidth="1"/>
+    <col min="2" max="2" width="13.140625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" ht="56.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="42" t="s">
+        <v>44</v>
+      </c>
+      <c r="B1" s="45" t="s">
+        <v>45</v>
+      </c>
+      <c r="C1" s="44"/>
+      <c r="D1" s="44"/>
+      <c r="E1" s="46"/>
+    </row>
+    <row r="2" spans="1:5" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="43"/>
+      <c r="B2" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="A3" s="34" t="s">
+        <v>50</v>
+      </c>
+      <c r="B3" s="33">
+        <v>5</v>
+      </c>
+      <c r="C3" s="33">
+        <v>4</v>
+      </c>
+      <c r="D3" s="33" t="s">
+        <v>31</v>
+      </c>
+      <c r="E3" s="33" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" ht="38.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="B4" s="29"/>
+      <c r="C4" s="29"/>
+      <c r="D4" s="29"/>
+      <c r="E4" s="29"/>
+    </row>
+    <row r="5" spans="1:5" ht="38.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="B5" s="48" t="s">
+        <v>31</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="D5" s="1">
+        <v>3</v>
+      </c>
+      <c r="E5" s="1">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" ht="38.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="5" t="s">
+        <v>53</v>
+      </c>
+      <c r="B6" s="1">
+        <v>2</v>
+      </c>
+      <c r="C6" s="1">
+        <v>2</v>
+      </c>
+      <c r="D6" s="1">
+        <v>2</v>
+      </c>
+      <c r="E6" s="1">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="5" t="s">
+        <v>54</v>
+      </c>
+      <c r="B7" s="1">
+        <v>15</v>
+      </c>
+      <c r="C7" s="1">
+        <v>12</v>
+      </c>
+      <c r="D7" s="1">
+        <v>8</v>
+      </c>
+      <c r="E7" s="1">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="B8" s="1">
+        <v>1</v>
+      </c>
+      <c r="C8" s="1">
+        <v>1</v>
+      </c>
+      <c r="D8" s="1">
+        <v>1</v>
+      </c>
+      <c r="E8" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" ht="38.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A9" s="5" t="s">
+        <v>56</v>
+      </c>
+      <c r="B9" s="1">
+        <v>2</v>
+      </c>
+      <c r="C9" s="1">
+        <v>2</v>
+      </c>
+      <c r="D9" s="1">
+        <v>2</v>
+      </c>
+      <c r="E9" s="1">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A10" s="5" t="s">
+        <v>57</v>
+      </c>
+      <c r="B10" s="1">
+        <v>1</v>
+      </c>
+      <c r="C10" s="1">
+        <v>1</v>
+      </c>
+      <c r="D10" s="1">
+        <v>1</v>
+      </c>
+      <c r="E10" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A11" s="5" t="s">
+        <v>58</v>
+      </c>
+      <c r="B11" s="1">
+        <v>1</v>
+      </c>
+      <c r="C11" s="1">
+        <v>1</v>
+      </c>
+      <c r="D11" s="1">
+        <v>1</v>
+      </c>
+      <c r="E11" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" ht="38.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A12" s="5" t="s">
+        <v>59</v>
+      </c>
+      <c r="B12" s="1">
+        <v>2</v>
+      </c>
+      <c r="C12" s="1">
+        <v>2</v>
+      </c>
+      <c r="D12" s="1">
+        <v>2</v>
+      </c>
+      <c r="E12" s="1">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A13" s="47"/>
+    </row>
+    <row r="14" spans="1:5" ht="87" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A14" s="33" t="s">
+        <v>33</v>
+      </c>
+      <c r="B14" s="30" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" ht="18.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A15" s="29"/>
+      <c r="B15" s="1">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A16" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="B16" s="1">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" ht="38.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A17" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="B17" s="1">
+        <v>5600</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" ht="38.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A18" s="5" t="s">
+        <v>37</v>
+      </c>
+      <c r="B18" s="1">
+        <v>850</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" ht="40.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A19" s="5" t="s">
+        <v>38</v>
+      </c>
+      <c r="B19" s="1">
+        <v>1275</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="7">
+    <mergeCell ref="A14:A15"/>
+    <mergeCell ref="A1:A2"/>
+    <mergeCell ref="B1:E1"/>
+    <mergeCell ref="B3:B4"/>
+    <mergeCell ref="C3:C4"/>
+    <mergeCell ref="D3:D4"/>
+    <mergeCell ref="E3:E4"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>